<commit_message>
Clarifie l'impact avant/après des actions et corrige MAC-018
</commit_message>
<xml_diff>
--- a/data_suivi/suivi_suggestions.xlsx
+++ b/data_suivi/suivi_suggestions.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Macro MAC-018 : réglage intensité/mode diffusion via l'app — adoptée par l'équipe (67% des tickets) mais CSAT quasi inchangé (3.51 -&gt; 3.44) : le réglage app ne résout pas le problème pour une partie des clients, la cause est probablement matérielle (à creuser avec le produit).</t>
+          <t>Macro MAC-018 : réglage intensité/mode diffusion via l'app, mis en place pour tenter de réduire les réclamations liées à un parfum délivré en excès. Hypothèse de l'équipe au moment de l'action : le réglage applicatif ne suffit probablement pas à couvrir tous les cas, la cause étant possiblement matérielle (à creuser avec le produit).</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>notes : libre (ex : lien vers la macro, qui l'a créée...).</t>
+          <t>notes : libre (ex : lien vers la macro, qui l'a créée...). Ne pas y saisir de KPI ou de valeurs avant/après calculables par Emyria (CSAT, volumes, taux) : ces valeurs sont produites automatiquement à partir de date_action.</t>
         </is>
       </c>
     </row>

</xml_diff>